<commit_message>
v445.12.0: Startup-Gründer und geprüfte Schnittflug-Akte veröffentlichen
</commit_message>
<xml_diff>
--- a/testakten/startup-gruender-schnittflug-berlin/50_CapTable_Gruendung_und_Finanzierungsoptionen.xlsx
+++ b/testakten/startup-gruender-schnittflug-berlin/50_CapTable_Gruendung_und_Finanzierungsoptionen.xlsx
@@ -2,16 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cap Table" sheetId="1" r:id="Rcb0a8e1fec5d44c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runden" sheetId="2" r:id="Rab3ca2ed547745b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Virtueller Pool" sheetId="3" r:id="R7f36c41ed516440e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eingaben" sheetId="4" r:id="Re89957ef6a524b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cap Table" sheetId="1" r:id="Rf50ad353dc234887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runden" sheetId="2" r:id="R378654e136614f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Virtueller Pool" sheetId="3" r:id="Rbf2a9f7fda894005"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eingaben" sheetId="4" r:id="Rd03eeb96fe9544fb"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="_xlnm.Print_Area" localSheetId="0">'Cap Table'!$B$2:$J$27</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="0">'Cap Table'!$6:$6</x:definedName>
     <x:definedName name="_xlnm.Print_Area" localSheetId="1">'Runden'!$B$2:$G$30</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="1">'Runden'!$6:$6</x:definedName>
     <x:definedName name="_xlnm.Print_Area" localSheetId="2">'Virtueller Pool'!$B$2:$F$25</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="2">'Virtueller Pool'!$6:$6</x:definedName>
     <x:definedName name="_xlnm.Print_Area" localSheetId="3">'Eingaben'!$B$2:$G$31</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="3">'Eingaben'!$18:$18</x:definedName>
   </x:definedNames>
 </x:workbook>
 </file>
@@ -1819,10 +1823,10 @@
   <x:cols>
     <x:col min="1" max="1" width="2" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="36.66999816894531" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="17.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="17.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -2794,5 +2798,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
   <x:pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <x:rowBreaks count="1" manualBreakCount="1">
+    <x:brk id="17" min="0" max="16383" man="1"/>
+  </x:rowBreaks>
 </x:worksheet>
 </file>
</xml_diff>